<commit_message>
ci: actualizar pipeline y persistencia de reportes JSON para dashboard
</commit_message>
<xml_diff>
--- a/excel-dashboard/QA_Executive_Dashboard.xlsx
+++ b/excel-dashboard/QA_Executive_Dashboard.xlsx
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="C2" s="11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D2" s="11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E2" s="11" t="n">
         <v>0</v>
@@ -991,7 +991,7 @@
         <v/>
       </c>
       <c r="H2" s="13" t="n">
-        <v>10150</v>
+        <v>6604</v>
       </c>
     </row>
     <row r="3">
@@ -1006,10 +1006,10 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D3" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3" s="11" t="n">
         <v>0</v>
@@ -1022,7 +1022,7 @@
         <v/>
       </c>
       <c r="H3" s="13" t="n">
-        <v>7412</v>
+        <v>6069</v>
       </c>
     </row>
     <row r="4">
@@ -1037,10 +1037,10 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" s="11" t="n">
         <v>0</v>
@@ -1053,7 +1053,7 @@
         <v/>
       </c>
       <c r="H4" s="13" t="n">
-        <v>9536</v>
+        <v>4434</v>
       </c>
     </row>
     <row r="5">
@@ -1068,10 +1068,10 @@
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" s="11" t="n">
         <v>0</v>
@@ -1084,7 +1084,7 @@
         <v/>
       </c>
       <c r="H5" s="13" t="n">
-        <v>3507</v>
+        <v>1850</v>
       </c>
     </row>
     <row r="6">
@@ -1099,10 +1099,10 @@
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D6" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" s="11" t="n">
         <v>0</v>
@@ -1115,7 +1115,7 @@
         <v/>
       </c>
       <c r="H6" s="13" t="n">
-        <v>3680</v>
+        <v>1645</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
feat: add QA Executive Dashboard Excel spreadsheet
</commit_message>
<xml_diff>
--- a/excel-dashboard/QA_Executive_Dashboard.xlsx
+++ b/excel-dashboard/QA_Executive_Dashboard.xlsx
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="C2" s="11" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D2" s="11" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E2" s="11" t="n">
         <v>0</v>
@@ -991,7 +991,7 @@
         <v/>
       </c>
       <c r="H2" s="13" t="n">
-        <v>6604</v>
+        <v>1456</v>
       </c>
     </row>
     <row r="3">
@@ -1006,10 +1006,10 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D3" s="11" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E3" s="11" t="n">
         <v>0</v>
@@ -1022,7 +1022,7 @@
         <v/>
       </c>
       <c r="H3" s="13" t="n">
-        <v>6069</v>
+        <v>640</v>
       </c>
     </row>
     <row r="4">
@@ -1037,10 +1037,10 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D4" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" s="11" t="n">
         <v>0</v>
@@ -1053,7 +1053,7 @@
         <v/>
       </c>
       <c r="H4" s="13" t="n">
-        <v>4434</v>
+        <v>2793</v>
       </c>
     </row>
     <row r="5">
@@ -1068,10 +1068,10 @@
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" s="11" t="n">
         <v>0</v>
@@ -1084,7 +1084,7 @@
         <v/>
       </c>
       <c r="H5" s="13" t="n">
-        <v>1850</v>
+        <v>2236</v>
       </c>
     </row>
     <row r="6">
@@ -1099,10 +1099,10 @@
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" s="11" t="n">
         <v>0</v>
@@ -1115,7 +1115,7 @@
         <v/>
       </c>
       <c r="H6" s="13" t="n">
-        <v>1645</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="7">

</xml_diff>